<commit_message>
Update LD annotation to WMtz
</commit_message>
<xml_diff>
--- a/processed-data/21_Xenium/Bansky_cluster_notes.xlsx
+++ b/processed-data/21_Xenium/Bansky_cluster_notes.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/8j/ftgpc01j3vx744_jxfrp_1rc0000gn/T/ch.sudo.cyberduck/editor-d7bf19b0-e05b-4a16-ab05-9cae49e74e86/dcs05/lieber/marmaypag/LFF_spatialERC_LIBD4140/LFF_spatial_ERC/processed-data/21_Xenium/111479615/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/8j/ftgpc01j3vx744_jxfrp_1rc0000gn/T/ch.sudo.cyberduck/editor-d7bf19b0-e05b-4a16-ab05-9cae49e74e86/dcs05/lieber/marmaypag/LFF_spatialERC_LIBD4140/LFF_spatial_ERC/processed-data/21_Xenium/94586280/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8CE5118-A387-4747-8851-8BC4893115D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D821C05-0B6D-CC41-9AD6-C6988B66324C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="41000" yWindow="2180" windowWidth="27640" windowHeight="16680" xr2:uid="{A7AE8A42-3C01-994B-8469-596FAD069385}"/>
   </bookViews>
@@ -53,9 +53,6 @@
     <t>L2.3</t>
   </si>
   <si>
-    <t>LD</t>
-  </si>
-  <si>
     <t>Inhib</t>
   </si>
   <si>
@@ -84,6 +81,9 @@
   </si>
   <si>
     <t>Xenium_k9</t>
+  </si>
+  <si>
+    <t>WMtz</t>
   </si>
 </sst>
 </file>
@@ -532,10 +532,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -546,7 +546,7 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -557,7 +557,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -568,7 +568,7 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -579,12 +579,12 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B6" s="9">
         <v>8</v>
@@ -592,18 +592,18 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="5">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8" s="6">
         <v>1</v>
@@ -611,7 +611,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="2">
         <v>9</v>
@@ -619,18 +619,18 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="1">
         <v>2</v>
       </c>
       <c r="C10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="1">
         <v>2</v>

</xml_diff>